<commit_message>
chore(pyhelix): tighten encoding tests and example console setup
Also restores events.xlsx create_event to boolean cells, which the row
append had rewritten as strings.
</commit_message>
<xml_diff>
--- a/libs/pyhelix/examples/dataset/events.xlsx
+++ b/libs/pyhelix/examples/dataset/events.xlsx
@@ -499,10 +499,8 @@
 </t>
         </is>
       </c>
-      <c r="L2" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L2" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3" ht="61.15" customHeight="1" s="5">
@@ -559,10 +557,8 @@
 </t>
         </is>
       </c>
-      <c r="L3" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L3" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4" ht="61.15" customHeight="1" s="5">
@@ -619,10 +615,8 @@
 </t>
         </is>
       </c>
-      <c r="L4" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L4" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5" ht="61.15" customHeight="1" s="5">
@@ -679,10 +673,8 @@
 </t>
         </is>
       </c>
-      <c r="L5" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L5" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="61.15" customHeight="1" s="5">
@@ -739,10 +731,8 @@
 </t>
         </is>
       </c>
-      <c r="L6" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L6" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7" ht="61.15" customHeight="1" s="5">
@@ -799,10 +789,8 @@
 </t>
         </is>
       </c>
-      <c r="L7" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L7" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8" ht="61.15" customHeight="1" s="5">
@@ -859,10 +847,8 @@
 </t>
         </is>
       </c>
-      <c r="L8" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L8" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9" ht="61.15" customHeight="1" s="5">
@@ -919,10 +905,8 @@
 </t>
         </is>
       </c>
-      <c r="L9" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L9" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10" ht="61.15" customHeight="1" s="5">
@@ -979,10 +963,8 @@
 </t>
         </is>
       </c>
-      <c r="L10" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L10" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="11" ht="61.15" customHeight="1" s="5">
@@ -1039,10 +1021,8 @@
 </t>
         </is>
       </c>
-      <c r="L11" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L11" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="12" ht="61.15" customHeight="1" s="5">
@@ -1099,10 +1079,8 @@
 </t>
         </is>
       </c>
-      <c r="L12" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L12" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="61.15" customHeight="1" s="5">
@@ -1159,10 +1137,8 @@
 </t>
         </is>
       </c>
-      <c r="L13" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L13" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14" ht="61.15" customHeight="1" s="5">
@@ -1219,10 +1195,8 @@
 </t>
         </is>
       </c>
-      <c r="L14" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L14" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="15" ht="61.15" customHeight="1" s="5">
@@ -1279,10 +1253,8 @@
 </t>
         </is>
       </c>
-      <c r="L15" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L15" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16" ht="61.15" customHeight="1" s="5">
@@ -1339,10 +1311,8 @@
 </t>
         </is>
       </c>
-      <c r="L16" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L16" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17" ht="61.15" customHeight="1" s="5">
@@ -1399,10 +1369,8 @@
 </t>
         </is>
       </c>
-      <c r="L17" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L17" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="18" ht="61.15" customHeight="1" s="5">
@@ -1459,10 +1427,8 @@
 </t>
         </is>
       </c>
-      <c r="L18" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L18" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="19" ht="61.15" customHeight="1" s="5">
@@ -1519,10 +1485,8 @@
 </t>
         </is>
       </c>
-      <c r="L19" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L19" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="20" ht="61.15" customHeight="1" s="5">
@@ -1579,10 +1543,8 @@
 </t>
         </is>
       </c>
-      <c r="L20" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L20" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="21" ht="61.15" customHeight="1" s="5">
@@ -1639,10 +1601,8 @@
 </t>
         </is>
       </c>
-      <c r="L21" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L21" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="22" ht="61.15" customHeight="1" s="5">
@@ -1699,10 +1659,8 @@
 </t>
         </is>
       </c>
-      <c r="L22" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L22" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="23" ht="61.15" customHeight="1" s="5">
@@ -1759,10 +1717,8 @@
 </t>
         </is>
       </c>
-      <c r="L23" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L23" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="24" ht="61.15" customHeight="1" s="5">
@@ -1819,10 +1775,8 @@
 </t>
         </is>
       </c>
-      <c r="L24" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L24" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="25" ht="61.15" customHeight="1" s="5">
@@ -1879,10 +1833,8 @@
 </t>
         </is>
       </c>
-      <c r="L25" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L25" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="26" ht="61.15" customHeight="1" s="5">
@@ -1939,10 +1891,8 @@
 </t>
         </is>
       </c>
-      <c r="L26" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L26" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="27" ht="61.15" customHeight="1" s="5">
@@ -1999,10 +1949,8 @@
 </t>
         </is>
       </c>
-      <c r="L27" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L27" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="28" ht="61.15" customHeight="1" s="5">
@@ -2059,10 +2007,8 @@
 </t>
         </is>
       </c>
-      <c r="L28" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L28" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="29" ht="61.15" customHeight="1" s="5">
@@ -2119,10 +2065,8 @@
 </t>
         </is>
       </c>
-      <c r="L29" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L29" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="30" ht="61.15" customHeight="1" s="5">
@@ -2179,10 +2123,8 @@
 </t>
         </is>
       </c>
-      <c r="L30" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L30" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="31" ht="61.15" customHeight="1" s="5">
@@ -2239,10 +2181,8 @@
 </t>
         </is>
       </c>
-      <c r="L31" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L31" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="32" ht="61.15" customHeight="1" s="5">
@@ -2299,10 +2239,8 @@
 </t>
         </is>
       </c>
-      <c r="L32" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L32" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="33" ht="61.15" customHeight="1" s="5">
@@ -2359,10 +2297,8 @@
 </t>
         </is>
       </c>
-      <c r="L33" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L33" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="34" ht="61.15" customHeight="1" s="5">
@@ -2419,10 +2355,8 @@
 </t>
         </is>
       </c>
-      <c r="L34" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L34" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="35" ht="61.15" customHeight="1" s="5">
@@ -2479,10 +2413,8 @@
 </t>
         </is>
       </c>
-      <c r="L35" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L35" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="36" ht="61.15" customHeight="1" s="5">
@@ -2539,10 +2471,8 @@
 </t>
         </is>
       </c>
-      <c r="L36" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L36" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="37" ht="61.15" customHeight="1" s="5">
@@ -2599,10 +2529,8 @@
 </t>
         </is>
       </c>
-      <c r="L37" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L37" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="38" ht="61.15" customHeight="1" s="5">
@@ -2659,10 +2587,8 @@
 </t>
         </is>
       </c>
-      <c r="L38" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L38" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="39" ht="61.15" customHeight="1" s="5">
@@ -2719,10 +2645,8 @@
 </t>
         </is>
       </c>
-      <c r="L39" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L39" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="40" ht="61.15" customHeight="1" s="5">
@@ -2779,10 +2703,8 @@
 </t>
         </is>
       </c>
-      <c r="L40" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L40" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="41" ht="61.15" customHeight="1" s="5">
@@ -2839,10 +2761,8 @@
 </t>
         </is>
       </c>
-      <c r="L41" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L41" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="42" ht="61.15" customHeight="1" s="5">
@@ -2899,10 +2819,8 @@
 </t>
         </is>
       </c>
-      <c r="L42" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L42" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="43" ht="61.15" customHeight="1" s="5">
@@ -2959,10 +2877,8 @@
 </t>
         </is>
       </c>
-      <c r="L43" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L43" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="44" ht="61.15" customHeight="1" s="5">
@@ -3019,10 +2935,8 @@
 </t>
         </is>
       </c>
-      <c r="L44" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L44" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="45" ht="61.15" customHeight="1" s="5">
@@ -3079,10 +2993,8 @@
 </t>
         </is>
       </c>
-      <c r="L45" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L45" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="46" ht="61.15" customHeight="1" s="5">
@@ -3139,10 +3051,8 @@
 </t>
         </is>
       </c>
-      <c r="L46" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L46" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="47" ht="61.15" customHeight="1" s="5">
@@ -3199,10 +3109,8 @@
 </t>
         </is>
       </c>
-      <c r="L47" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L47" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="48" ht="61.15" customHeight="1" s="5">
@@ -3259,10 +3167,8 @@
 </t>
         </is>
       </c>
-      <c r="L48" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L48" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="49" ht="61.15" customHeight="1" s="5">
@@ -3319,10 +3225,8 @@
 </t>
         </is>
       </c>
-      <c r="L49" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L49" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="50" ht="61.15" customHeight="1" s="5">
@@ -3379,10 +3283,8 @@
 </t>
         </is>
       </c>
-      <c r="L50" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L50" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="51" ht="61.15" customHeight="1" s="5">
@@ -3439,10 +3341,8 @@
 </t>
         </is>
       </c>
-      <c r="L51" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L51" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="52" ht="61.15" customHeight="1" s="5">
@@ -3499,10 +3399,8 @@
 </t>
         </is>
       </c>
-      <c r="L52" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L52" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="53" ht="61.15" customHeight="1" s="5">
@@ -3559,10 +3457,8 @@
 </t>
         </is>
       </c>
-      <c r="L53" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L53" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="54" ht="61.15" customHeight="1" s="5">
@@ -3619,10 +3515,8 @@
 </t>
         </is>
       </c>
-      <c r="L54" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L54" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="55" ht="61.15" customHeight="1" s="5">
@@ -3679,10 +3573,8 @@
 </t>
         </is>
       </c>
-      <c r="L55" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L55" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="56" ht="61.15" customHeight="1" s="5">
@@ -3739,10 +3631,8 @@
 </t>
         </is>
       </c>
-      <c r="L56" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L56" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="57" ht="61.15" customHeight="1" s="5">
@@ -3799,10 +3689,8 @@
 </t>
         </is>
       </c>
-      <c r="L57" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L57" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="58" ht="61.15" customHeight="1" s="5">
@@ -3859,10 +3747,8 @@
 </t>
         </is>
       </c>
-      <c r="L58" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L58" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="59" ht="61.15" customHeight="1" s="5">
@@ -3919,10 +3805,8 @@
 </t>
         </is>
       </c>
-      <c r="L59" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L59" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="60" ht="61.15" customHeight="1" s="5">
@@ -3979,10 +3863,8 @@
 </t>
         </is>
       </c>
-      <c r="L60" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L60" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="61" ht="61.15" customHeight="1" s="5">
@@ -4039,10 +3921,8 @@
 </t>
         </is>
       </c>
-      <c r="L61" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L61" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="62" ht="61.15" customHeight="1" s="5">
@@ -4099,10 +3979,8 @@
 </t>
         </is>
       </c>
-      <c r="L62" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L62" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="63" ht="61.15" customHeight="1" s="5">
@@ -4159,10 +4037,8 @@
 </t>
         </is>
       </c>
-      <c r="L63" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L63" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="64" ht="61.15" customHeight="1" s="5">
@@ -4219,10 +4095,8 @@
 </t>
         </is>
       </c>
-      <c r="L64" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L64" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="65" ht="61.15" customHeight="1" s="5">
@@ -4279,10 +4153,8 @@
 </t>
         </is>
       </c>
-      <c r="L65" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L65" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="66" ht="61.15" customHeight="1" s="5">
@@ -4339,10 +4211,8 @@
 </t>
         </is>
       </c>
-      <c r="L66" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L66" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="67" ht="61.15" customHeight="1" s="5">
@@ -4399,10 +4269,8 @@
 </t>
         </is>
       </c>
-      <c r="L67" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L67" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="68" ht="61.15" customHeight="1" s="5">
@@ -4459,10 +4327,8 @@
 </t>
         </is>
       </c>
-      <c r="L68" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L68" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="69" ht="61.15" customHeight="1" s="5">
@@ -4519,10 +4385,8 @@
 </t>
         </is>
       </c>
-      <c r="L69" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L69" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="70" ht="61.15" customHeight="1" s="5">
@@ -4579,10 +4443,8 @@
 </t>
         </is>
       </c>
-      <c r="L70" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L70" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="71" ht="61.15" customHeight="1" s="5">
@@ -4639,10 +4501,8 @@
 </t>
         </is>
       </c>
-      <c r="L71" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L71" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="72" ht="61.15" customHeight="1" s="5">
@@ -4699,10 +4559,8 @@
 </t>
         </is>
       </c>
-      <c r="L72" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L72" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="73" ht="61.15" customHeight="1" s="5">
@@ -4759,10 +4617,8 @@
 </t>
         </is>
       </c>
-      <c r="L73" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L73" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="74" ht="61.15" customHeight="1" s="5">
@@ -4819,10 +4675,8 @@
 </t>
         </is>
       </c>
-      <c r="L74" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L74" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="75" ht="61.15" customHeight="1" s="5">
@@ -4879,10 +4733,8 @@
 </t>
         </is>
       </c>
-      <c r="L75" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L75" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="76" ht="61.15" customHeight="1" s="5">
@@ -4939,10 +4791,8 @@
 </t>
         </is>
       </c>
-      <c r="L76" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L76" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="77" ht="61.15" customHeight="1" s="5">
@@ -4999,10 +4849,8 @@
 </t>
         </is>
       </c>
-      <c r="L77" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L77" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="78" ht="61.15" customHeight="1" s="5">
@@ -5059,10 +4907,8 @@
 </t>
         </is>
       </c>
-      <c r="L78" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L78" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="79" ht="61.15" customHeight="1" s="5">
@@ -5119,10 +4965,8 @@
 </t>
         </is>
       </c>
-      <c r="L79" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L79" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="80" ht="61.15" customHeight="1" s="5">
@@ -5179,10 +5023,8 @@
 </t>
         </is>
       </c>
-      <c r="L80" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L80" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="81" ht="61.15" customHeight="1" s="5">
@@ -5239,10 +5081,8 @@
 </t>
         </is>
       </c>
-      <c r="L81" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L81" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="82" ht="61.15" customHeight="1" s="5">
@@ -5299,10 +5139,8 @@
 </t>
         </is>
       </c>
-      <c r="L82" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L82" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="83" ht="61.15" customHeight="1" s="5">
@@ -5359,10 +5197,8 @@
 </t>
         </is>
       </c>
-      <c r="L83" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L83" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="84" ht="61.15" customHeight="1" s="5">
@@ -5419,10 +5255,8 @@
 </t>
         </is>
       </c>
-      <c r="L84" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L84" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="85" ht="61.15" customHeight="1" s="5">
@@ -5479,10 +5313,8 @@
 </t>
         </is>
       </c>
-      <c r="L85" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L85" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="86" ht="61.15" customHeight="1" s="5">
@@ -5539,10 +5371,8 @@
 </t>
         </is>
       </c>
-      <c r="L86" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L86" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="87" ht="61.15" customHeight="1" s="5">
@@ -5599,10 +5429,8 @@
 </t>
         </is>
       </c>
-      <c r="L87" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L87" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="88" ht="61.15" customHeight="1" s="5">
@@ -5659,10 +5487,8 @@
 </t>
         </is>
       </c>
-      <c r="L88" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L88" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="89" ht="61.15" customHeight="1" s="5">
@@ -5719,10 +5545,8 @@
 </t>
         </is>
       </c>
-      <c r="L89" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L89" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="90" ht="61.15" customHeight="1" s="5">
@@ -5779,10 +5603,8 @@
 </t>
         </is>
       </c>
-      <c r="L90" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L90" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="91" ht="61.15" customHeight="1" s="5">
@@ -5839,10 +5661,8 @@
 </t>
         </is>
       </c>
-      <c r="L91" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L91" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="92" ht="61.15" customHeight="1" s="5">
@@ -5899,10 +5719,8 @@
 </t>
         </is>
       </c>
-      <c r="L92" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L92" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="93" ht="61.15" customHeight="1" s="5">
@@ -5959,10 +5777,8 @@
 </t>
         </is>
       </c>
-      <c r="L93" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L93" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="94" ht="61.15" customHeight="1" s="5">
@@ -6019,10 +5835,8 @@
 </t>
         </is>
       </c>
-      <c r="L94" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L94" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="95" ht="61.15" customHeight="1" s="5">
@@ -6079,10 +5893,8 @@
 </t>
         </is>
       </c>
-      <c r="L95" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L95" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="96" ht="61.15" customHeight="1" s="5">
@@ -6139,10 +5951,8 @@
 </t>
         </is>
       </c>
-      <c r="L96" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L96" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="97" ht="61.15" customHeight="1" s="5">
@@ -6199,10 +6009,8 @@
 </t>
         </is>
       </c>
-      <c r="L97" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L97" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="98" ht="61.15" customHeight="1" s="5">
@@ -6259,10 +6067,8 @@
 </t>
         </is>
       </c>
-      <c r="L98" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L98" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="99" ht="61.15" customHeight="1" s="5">
@@ -6319,10 +6125,8 @@
 </t>
         </is>
       </c>
-      <c r="L99" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L99" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="100" ht="61.15" customHeight="1" s="5">
@@ -6379,10 +6183,8 @@
 </t>
         </is>
       </c>
-      <c r="L100" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L100" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="101" ht="61.15" customHeight="1" s="5">
@@ -6439,10 +6241,8 @@
 </t>
         </is>
       </c>
-      <c r="L101" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L101" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="102" ht="61.15" customHeight="1" s="5">
@@ -6499,10 +6299,8 @@
 </t>
         </is>
       </c>
-      <c r="L102" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L102" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="103" ht="61.15" customHeight="1" s="5">
@@ -6559,10 +6357,8 @@
 </t>
         </is>
       </c>
-      <c r="L103" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L103" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="104" ht="61.15" customHeight="1" s="5">
@@ -6619,10 +6415,8 @@
 </t>
         </is>
       </c>
-      <c r="L104" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L104" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="105" ht="61.15" customHeight="1" s="5">
@@ -6679,10 +6473,8 @@
 </t>
         </is>
       </c>
-      <c r="L105" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L105" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="106" ht="61.15" customHeight="1" s="5">
@@ -6739,10 +6531,8 @@
 </t>
         </is>
       </c>
-      <c r="L106" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L106" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="107" ht="61.15" customHeight="1" s="5">
@@ -6799,10 +6589,8 @@
 </t>
         </is>
       </c>
-      <c r="L107" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L107" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="108" ht="61.15" customHeight="1" s="5">
@@ -6859,10 +6647,8 @@
 </t>
         </is>
       </c>
-      <c r="L108" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L108" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="109" ht="61.15" customHeight="1" s="5">
@@ -6919,59 +6705,57 @@
 </t>
         </is>
       </c>
-      <c r="L109" s="8" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L109" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="110">
-      <c r="A110" t="inlineStr">
+      <c r="A110" s="8" t="inlineStr">
         <is>
           <t>3ed97a61-3ba2-5940-8f9b-387c00e26b6a</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="B110" s="8" t="inlineStr">
         <is>
           <t>Afghanistan: Mixed disasters - Kandahār (قندهار) - 15/09/2025</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>Disaster</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr">
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>Disaster</t>
+        </is>
+      </c>
+      <c r="D110" s="8" t="inlineStr">
         <is>
           <t>Mixed disasters</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
+      <c r="E110" s="8" t="inlineStr">
         <is>
           <t>Afghanistan</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
+      <c r="F110" s="8" t="inlineStr">
         <is>
           <t>2025-09-15</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="H110" t="inlineStr">
+      <c r="G110" s="8" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="H110" s="8" t="inlineStr">
         <is>
           <t>2025-09-15</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="K110" t="inlineStr">
+      <c r="I110" s="8" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="K110" s="8" t="inlineStr">
         <is>
           <t>This is an event created based on data received for Afghanistan.
 **Analysis**
@@ -6979,59 +6763,57 @@
 On 15 September, mixed disasters displaced 4.0 households in Spīn Bůldąk.</t>
         </is>
       </c>
-      <c r="L110" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L110" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr">
+      <c r="A111" s="8" t="inlineStr">
         <is>
           <t>80289cce-d973-5eb2-9153-956a79e89371</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="B111" s="8" t="inlineStr">
         <is>
           <t>Haiti: Mixed disasters - Ouanaminthe‗ (Nord-Est) - 16/09/2025</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>Disaster</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>Disaster</t>
+        </is>
+      </c>
+      <c r="D111" s="8" t="inlineStr">
         <is>
           <t>Mixed disasters</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
+      <c r="E111" s="8" t="inlineStr">
         <is>
           <t>Haiti</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr">
+      <c r="F111" s="8" t="inlineStr">
         <is>
           <t>2025-09-16</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr">
+      <c r="G111" s="8" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="H111" s="8" t="inlineStr">
         <is>
           <t>2025-09-16</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="K111" t="inlineStr">
+      <c r="I111" s="8" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="K111" s="8" t="inlineStr">
         <is>
           <t>This is an event created based on data received for Haiti.
 **Analysis**
@@ -7039,59 +6821,57 @@
 On 16 September, mixed disasters displaced 2.0 households.</t>
         </is>
       </c>
-      <c r="L111" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L111" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="112">
-      <c r="A112" t="inlineStr">
+      <c r="A112" s="8" t="inlineStr">
         <is>
           <t>c6e61102-e62d-5383-b78b-5a4a48007c99</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="B112" s="8" t="inlineStr">
         <is>
           <t>Iraq: Mixed disasters - Ḩadīthah (Al-Anbār) - 17/09/2025</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>Disaster</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t>Disaster</t>
+        </is>
+      </c>
+      <c r="D112" s="8" t="inlineStr">
         <is>
           <t>Mixed disasters</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
+      <c r="E112" s="8" t="inlineStr">
         <is>
           <t>Iraq</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr">
+      <c r="F112" s="8" t="inlineStr">
         <is>
           <t>2025-09-17</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="H112" t="inlineStr">
+      <c r="G112" s="8" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="H112" s="8" t="inlineStr">
         <is>
           <t>2025-09-17</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="K112" t="inlineStr">
+      <c r="I112" s="8" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="K112" s="8" t="inlineStr">
         <is>
           <t>This is an event created based on data received for Iraq.
 **Analysis**
@@ -7099,59 +6879,57 @@
 On 17 September, mixed disasters displaced 3.0 households in Żumar.</t>
         </is>
       </c>
-      <c r="L112" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L112" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" t="inlineStr">
+      <c r="A113" s="8" t="inlineStr">
         <is>
           <t>4c74a367-3be5-5244-b2ce-1c9d2186e723</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
+      <c r="B113" s="8" t="inlineStr">
         <is>
           <t>Nepal: Mixed disasters - Kāthmān̄ḍaū (Bāgmatī) - 18/09/2025</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
-        <is>
-          <t>Disaster</t>
-        </is>
-      </c>
-      <c r="D113" t="inlineStr">
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>Disaster</t>
+        </is>
+      </c>
+      <c r="D113" s="8" t="inlineStr">
         <is>
           <t>Mixed disasters</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr">
+      <c r="E113" s="8" t="inlineStr">
         <is>
           <t>Nepal</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr">
+      <c r="F113" s="8" t="inlineStr">
         <is>
           <t>2025-09-18</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="H113" t="inlineStr">
+      <c r="G113" s="8" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="H113" s="8" t="inlineStr">
         <is>
           <t>2025-09-18</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="K113" t="inlineStr">
+      <c r="I113" s="8" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="K113" s="8" t="inlineStr">
         <is>
           <t>This is an event created based on data received for Nepal.
 **Analysis**
@@ -7159,59 +6937,57 @@
 On 18 September, mixed disasters displaced 5.0 households in Sindhupālcok.</t>
         </is>
       </c>
-      <c r="L113" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L113" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
+      <c r="A114" s="8" t="inlineStr">
         <is>
           <t>c09ca4f9-4323-5280-900a-a74014fef7c4</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B114" s="8" t="inlineStr">
         <is>
           <t>Palestine: Mixed disasters - Ṭūbās - 19/09/2025</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
-        <is>
-          <t>Disaster</t>
-        </is>
-      </c>
-      <c r="D114" t="inlineStr">
+      <c r="C114" s="8" t="inlineStr">
+        <is>
+          <t>Disaster</t>
+        </is>
+      </c>
+      <c r="D114" s="8" t="inlineStr">
         <is>
           <t>Mixed disasters</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
+      <c r="E114" s="8" t="inlineStr">
         <is>
           <t>Palestine</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr">
+      <c r="F114" s="8" t="inlineStr">
         <is>
           <t>2025-09-19</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="H114" t="inlineStr">
+      <c r="G114" s="8" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="H114" s="8" t="inlineStr">
         <is>
           <t>2025-09-19</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="K114" t="inlineStr">
+      <c r="I114" s="8" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="K114" s="8" t="inlineStr">
         <is>
           <t>This is an event created based on data received for Palestine.
 **Analysis**
@@ -7219,59 +6995,57 @@
 On 19 September, mixed disasters displaced 1.0 household in Mạsāfer Yaṭṭā.</t>
         </is>
       </c>
-      <c r="L114" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L114" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="115">
-      <c r="A115" t="inlineStr">
+      <c r="A115" s="8" t="inlineStr">
         <is>
           <t>334da407-202a-533f-bb5e-21c1b0a095c3</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B115" s="8" t="inlineStr">
         <is>
           <t>Yemen: Mixed disasters - Ḩajjah (ʿAbs) - 20/09/2025</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>Disaster</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
+      <c r="C115" s="8" t="inlineStr">
+        <is>
+          <t>Disaster</t>
+        </is>
+      </c>
+      <c r="D115" s="8" t="inlineStr">
         <is>
           <t>Mixed disasters</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr">
+      <c r="E115" s="8" t="inlineStr">
         <is>
           <t>Yemen</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr">
+      <c r="F115" s="8" t="inlineStr">
         <is>
           <t>2025-09-20</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="H115" t="inlineStr">
+      <c r="G115" s="8" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="H115" s="8" t="inlineStr">
         <is>
           <t>2025-09-20</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr">
-        <is>
-          <t>Day</t>
-        </is>
-      </c>
-      <c r="K115" t="inlineStr">
+      <c r="I115" s="8" t="inlineStr">
+        <is>
+          <t>Day</t>
+        </is>
+      </c>
+      <c r="K115" s="8" t="inlineStr">
         <is>
           <t>This is an event created based on data received for Yemen.
 **Analysis**
@@ -7279,10 +7053,8 @@
 On 20 September, mixed disasters displaced 6.0 households in Miʿyān and ʾAmrān.</t>
         </is>
       </c>
-      <c r="L115" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
+      <c r="L115" s="8" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>